<commit_message>
feat(schema): model the CIS Controls' structure, with no CIS text
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/cis_controls.xlsx
+++ b/project/excel/cis_controls.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CISControlsDocument" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CISControl" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Safeguard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CisControls" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CisControl" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CisSafeguard" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,38 +415,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>cis_version</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>publication_date</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>controls</t>
+          <t>cis_controls</t>
         </is>
       </c>
     </row>
@@ -461,13 +441,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>cis_control_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -477,27 +457,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>control_number</t>
+          <t>description</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>overview</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>why_critical</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>procedures_and_tools</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>safeguards</t>
+          <t>control_safeguards</t>
         </is>
       </c>
     </row>
@@ -512,13 +477,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>cis_safeguard_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -528,39 +493,34 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>safeguard_number</t>
+          <t>description</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>safeguard_asset_class</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>asset_type</t>
+          <t>safeguard_security_function</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>security_function</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>implementation_groups</t>
+          <t>safeguard_implementation_groups</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"DEVICES,SOFTWARE,DATA,USERS,NETWORK,DOCUMENTATION"</formula1>
+    </dataValidation>
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Devices,Software,Data,Users,Network,Documentation"</formula1>
+      <formula1>"GOVERN,IDENTIFY,PROTECT,DETECT,RESPOND,RECOVER"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Govern,Identify,Protect,Detect,Respond,Recover"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"IG1,IG2,IG3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>